<commit_message>
Update XLSX parser to handle material categories and grades
- Modified xlsx_parser.py to implement material grade detection logic, extracting concrete grades (e.g. B20, B35) from element names or object types when available
- Enhanced material aggregation to separate entries by grade, creating distinct rows for materials like "Concrete B35" vs "Concrete B20"
- Updated parsing logic to check multiple potential material columns including ExpCheck patterns
- Improved material classification by adding concrete-like material detection for proper grade appending
- Updated output format maintains same structure but now shows detailed material grades
- Updated materials_summary.json and materials_summary.xlsx reflect new granular material categorization with increased item count from 10 to 15 due to grade separation
- Added .gitignore rule for uploads directory to prevent temporary files from being tracked
</commit_message>
<xml_diff>
--- a/uploads/ac993931-a75e-432c-ad3a-cd24b6131463/materials_summary.xlsx
+++ b/uploads/ac993931-a75e-432c-ad3a-cd24b6131463/materials_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Сводка по элементам" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка по элементам" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -519,7 +519,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Бетон</t>
+          <t>Бетон В30</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -575,7 +575,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Бетон</t>
+          <t>Бетон В30</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -609,13 +609,13 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>119</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2987992.324</v>
+        <v>0.364</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>44171.162</v>
+        <v>8.449</v>
       </c>
     </row>
     <row r="7">
@@ -631,128 +631,258 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Не указан</t>
+          <t>Бетон В10</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>8869.183000000001</v>
+        <v>66230.083</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>5640.589</v>
+        <v>5278.995</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Проемы</t>
+          <t>Перекрытия</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>IfcOpeningElement</t>
+          <t>IfcSlab</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Не указан</t>
+          <t>Бетон В25</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>490</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>66</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>2258957.128</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>23970.997</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Прочие_элементы</t>
+          <t>Перекрытия</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>IfcBuildingElementProxy</t>
+          <t>IfcSlab</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Не указан</t>
+          <t>Бетон В30</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1291</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>21</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>272423.156</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10344.024</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Стены</t>
+          <t>Перекрытия</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>IfcWall</t>
+          <t>IfcSlab</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Бетон</t>
+          <t>Бетон В35</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1147</v>
+        <v>23</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2363579.814</v>
+        <v>390381.593</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>20253.419</v>
+        <v>4568.696</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Перекрытия</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>IfcSlab</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>8869.183000000001</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>5640.589</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Проемы</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>IfcOpeningElement</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>490</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Прочие_элементы</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>IfcBuildingElementProxy</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1291</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>Стены</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>IfcWall</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В30</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>984</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1752340.901</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>15738.991</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Стены</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>IfcWall</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В35</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>611238.9129999999</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>4514.428</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Стены</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>IfcWall</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Не указан</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D16" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E16" s="2" t="n">
         <v>30568.661</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F16" s="2" t="n">
         <v>2715.508</v>
       </c>
     </row>

</xml_diff>